<commit_message>
importation excel landmarks et fACP
</commit_message>
<xml_diff>
--- a/data/Date_landmarks_20essais.xlsx
+++ b/data/Date_landmarks_20essais.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN.RDS-PRET-0218\Desktop\Agrocampus Ouest\M2\Projet ingénieur\meteo_vs_rendement\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1DBEE1D-65E4-4CD6-896C-A32D99521B9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4775EFB4-BE81-46C8-B646-FA8603E4ECF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="49">
   <si>
     <t>RAGT14</t>
   </si>
@@ -183,6 +183,9 @@
   </si>
   <si>
     <t>YEAR</t>
+  </si>
+  <si>
+    <t>FIN_P1000</t>
   </si>
 </sst>
 </file>
@@ -505,7 +508,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="8" width="17.81640625" customWidth="1"/>
-    <col min="9" max="10" width="28.1796875" customWidth="1"/>
+    <col min="9" max="9" width="12.54296875" customWidth="1"/>
+    <col min="10" max="10" width="28.1796875" customWidth="1"/>
     <col min="11" max="11" width="16.7265625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -534,6 +538,9 @@
       <c r="H1" t="s">
         <v>44</v>
       </c>
+      <c r="I1" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
@@ -561,7 +568,9 @@
         <f t="shared" ref="H2:H21" si="0">_xlfn.DAYS(G2,F2)</f>
         <v>43</v>
       </c>
-      <c r="I2" s="1"/>
+      <c r="I2" s="1">
+        <v>40703</v>
+      </c>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
@@ -590,7 +599,9 @@
         <f t="shared" si="0"/>
         <v>49</v>
       </c>
-      <c r="I3" s="1"/>
+      <c r="I3" s="1">
+        <v>40718</v>
+      </c>
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -619,7 +630,9 @@
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="I4" s="1"/>
+      <c r="I4" s="1">
+        <v>41089</v>
+      </c>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -648,7 +661,9 @@
         <f>_xlfn.DAYS(G5,F5)</f>
         <v>49</v>
       </c>
-      <c r="I5" s="1"/>
+      <c r="I5" s="1">
+        <v>41461</v>
+      </c>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -677,7 +692,9 @@
         <f t="shared" si="0"/>
         <v>58</v>
       </c>
-      <c r="I6" s="1"/>
+      <c r="I6" s="1">
+        <v>41472</v>
+      </c>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -706,7 +723,9 @@
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
-      <c r="I7" s="1"/>
+      <c r="I7" s="1">
+        <v>41810</v>
+      </c>
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -735,7 +754,9 @@
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="I8" s="1"/>
+      <c r="I8" s="1">
+        <v>41818</v>
+      </c>
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -764,7 +785,9 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="I9" s="1"/>
+      <c r="I9" s="1">
+        <v>41819</v>
+      </c>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -793,7 +816,9 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="I10" s="1"/>
+      <c r="I10" s="1">
+        <v>41826</v>
+      </c>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -822,7 +847,9 @@
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="I11" s="1"/>
+      <c r="I11" s="1">
+        <v>42167</v>
+      </c>
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -851,7 +878,9 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="I12" s="1"/>
+      <c r="I12" s="1">
+        <v>42186</v>
+      </c>
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -880,7 +909,9 @@
         <f t="shared" si="0"/>
         <v>99</v>
       </c>
-      <c r="I13" s="1"/>
+      <c r="I13" s="1">
+        <v>42189</v>
+      </c>
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -909,7 +940,9 @@
         <f t="shared" si="0"/>
         <v>91</v>
       </c>
-      <c r="I14" s="1"/>
+      <c r="I14" s="1">
+        <v>42187</v>
+      </c>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -938,7 +971,9 @@
         <f t="shared" si="0"/>
         <v>97</v>
       </c>
-      <c r="I15" s="1"/>
+      <c r="I15" s="1">
+        <v>42193</v>
+      </c>
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -967,7 +1002,9 @@
         <f t="shared" si="0"/>
         <v>97</v>
       </c>
-      <c r="I16" s="1"/>
+      <c r="I16" s="1">
+        <v>42194</v>
+      </c>
       <c r="J16" s="1"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
@@ -996,7 +1033,9 @@
         <f t="shared" si="0"/>
         <v>92</v>
       </c>
-      <c r="I17" s="1"/>
+      <c r="I17" s="1">
+        <v>42184</v>
+      </c>
       <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
@@ -1025,7 +1064,9 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="I18" s="1"/>
+      <c r="I18" s="1">
+        <v>42547</v>
+      </c>
       <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
@@ -1054,7 +1095,9 @@
         <f t="shared" si="0"/>
         <v>61</v>
       </c>
-      <c r="I19" s="1"/>
+      <c r="I19" s="1">
+        <v>42911</v>
+      </c>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -1083,6 +1126,9 @@
         <f t="shared" si="0"/>
         <v>94</v>
       </c>
+      <c r="I20" s="1">
+        <v>43276</v>
+      </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
@@ -1109,6 +1155,9 @@
       <c r="H21">
         <f t="shared" si="0"/>
         <v>93</v>
+      </c>
+      <c r="I21" s="1">
+        <v>43280</v>
       </c>
     </row>
   </sheetData>

</xml_diff>